<commit_message>
Ajout vérification image, export façon Amazon, renommage de l'app
</commit_message>
<xml_diff>
--- a/sample_data/produits_demo.xlsx
+++ b/sample_data/produits_demo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,6 +442,11 @@
           <t>infos_produits</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>image_url</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -469,6 +474,7 @@
           <t>750ml, garde le froid 24h, sans BPA, anse de transport</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -496,6 +502,7 @@
           <t>bluetooth 5.3, autonomie 30h, reduction de bruit active, etanche ipx5</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -523,6 +530,7 @@
           <t>40 litres, impermeable, compartiment ordinateur, bretelles rembourrees</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -550,6 +558,7 @@
           <t>3 temperatures de couleur, variateur tactile, port usb integre</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -577,6 +586,7 @@
           <t>ralentit la prise alimentaire, facile a nettoyer, base antiderapante</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Images secondaires, champs obligatoires, thème sombre, historique de session
</commit_message>
<xml_diff>
--- a/sample_data/produits_demo.xlsx
+++ b/sample_data/produits_demo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,11 @@
           <t>image_url</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>images_secondaires</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -475,6 +480,7 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -503,6 +509,7 @@
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -531,6 +538,7 @@
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -559,6 +567,7 @@
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -587,6 +596,7 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>